<commit_message>
Add carousel-cards, columns-feature blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (11):
- .migration/project.json
- blocks/carousel-cards/carousel-cards.css
- blocks/carousel-cards/carousel-cards.js
- blocks/columns-feature/columns-feature.css
- styles/styles.css
- tools/importer/reports/import-natwest.report.xlsx
- tools/importer/reports/index.report.json
- tools/importer/reports/mortgages/first-time-buyers.report.json
- tools/importer/reports/personal/insurance.report.json
- tools/importer/reports/premier-banking.report.json
- tools/importer/reports/support-centre/contact-us.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-natwest.report.xlsx
+++ b/tools/importer/reports/import-natwest.report.xlsx
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-07-16T14:57:01.592Z</t>
+    <t>2026-07-29T07:47:26.250Z</t>
   </si>
   <si>
     <t>NatWest Online – Bank Accounts, Mortgages, Loans and Savings</t>
@@ -73,7 +73,7 @@
     <t>segment-landing</t>
   </si>
   <si>
-    <t>2026-07-16T14:57:29.879Z</t>
+    <t>2026-07-29T07:47:55.783Z</t>
   </si>
   <si>
     <t>Premier banking | NatWest</t>
@@ -94,7 +94,7 @@
     <t>product-detail</t>
   </si>
   <si>
-    <t>2026-07-16T14:57:23.816Z</t>
+    <t>2026-07-29T07:47:49.098Z</t>
   </si>
   <si>
     <t>Get a Mortgage Agreement in Principle (AIP) | Decision in Principle | NatWest</t>
@@ -115,7 +115,7 @@
     <t>product-overview</t>
   </si>
   <si>
-    <t>2026-07-16T14:57:14.818Z</t>
+    <t>2026-07-29T07:47:41.509Z</t>
   </si>
   <si>
     <t>Home Insurance | Buildings and Contents Insurance | NatWest</t>
@@ -136,7 +136,7 @@
     <t>content-article</t>
   </si>
   <si>
-    <t>2026-07-16T14:57:07.177Z</t>
+    <t>2026-07-29T07:47:33.985Z</t>
   </si>
   <si>
     <t>Contact Us | Customer Support | NatWest</t>

</xml_diff>